<commit_message>
Update Christopher Morris Kensei task bundle
</commit_message>
<xml_diff>
--- a/data/file_57.xlsx
+++ b/data/file_57.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="closed_archive" sheetId="1" r:id="R10792c138c8d45b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="closed_archive" sheetId="1" r:id="R03a5f7875a864743"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,13 +21,13 @@
     <x:font>
       <x:b/>
       <x:sz val="13"/>
-      <x:color rgb="1F1F1F"/>
+      <x:color rgb="FF1F1F1F"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FFFFFF"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
@@ -40,12 +40,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="EFE8DC"/>
+        <x:fgColor rgb="FFEFE8DC"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="6F6255"/>
+        <x:fgColor rgb="FF6F6255"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -285,7 +285,7 @@
         <x:v>318400</x:v>
       </x:c>
       <x:c r="E4" s="14" t="str">
-        <x:v>Archive only, not Prairie Valley</x:v>
+        <x:v>Closed renewal history</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>